<commit_message>
Finish live Legacy Wire 10112–10115; remove 10113 invented PPV.
Select Receipts already on 24187 / 24188+24191 / 24189+24190 / 24192.
Removed 10113 −$85 and +$170 PPV so Invoice_Amount hits PDF $2600.
10115 stays on TRANSFER AP with in-gate $0.30 rounding PPV.
10116 left HOLD. Outlook Entered in AI on Success. No Mail.Send.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-17-legacy-wire.xlsx
+++ b/runs/AP-run-2026-09-17-legacy-wire.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -42,6 +42,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -62,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -71,6 +76,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -561,12 +569,12 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>Success</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>HOLD (receipt): no matching leftover receipts selected on PO 59034 for Legacy Wire invoice #PS-INV104020. PDF merch=75-10-201007 19@41; selected=none. Do not first-open guess. Do not invent Success. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59034. Select Receipts 24187 19@41.0 on PO 59034. Invoice #=PS-INV104020 (exact PDF, not stripped). Fees=Freight Charge - Wholesale - In 250.0 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -599,7 +607,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
@@ -630,12 +638,12 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>Success</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>HOLD (receipt): no matching leftover receipts selected on PO 59030 for Legacy Wire invoice #PS-INV104019. PDF merch=A-02390-000 17@36; A-06809-000 27@44; selected=none. Do not first-open guess. Do not invent Success.  Live GET still has invented PPV [-85.0] with no receipts (Removed PUT rolled back). Treyce should delete that PPV. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59030. Select Receipts 24188 17@36.0; 24191 27@44.0 on PO 59030. Invoice #=PS-INV104019 (exact PDF, not stripped). Fees=Freight Charge - Wholesale - In 800.0 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -653,7 +661,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>-85.00</t>
+          <t>none</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -668,7 +676,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
@@ -699,12 +707,12 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>Success</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>HOLD (receipt): no matching leftover receipts selected on PO 59030 for Legacy Wire invoice #PS-INV104018. PDF merch=75-10-201007 9@41; 75-10-201007 17@41; selected=none. Do not first-open guess. Do not invent Success. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59030. Select Receipts 24189 9@41.0; 24190 17@41.0 on PO 59030. Invoice #=PS-INV104018 (exact PDF, not stripped). Fees=Freight Charge - Wholesale - In 371.42 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -737,7 +745,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
@@ -768,12 +776,12 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>Success</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>HOLD (receipt): no matching leftover receipts selected on PO 58977 for Legacy Wire invoice #PS-INV104015. PDF merch=75-21-101007 100@0.78; selected=none. Do not first-open guess. Do not invent Success. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set=58977. Select Receipts 24192 100@0.777 on PO 58977. Invoice #=PS-INV104015 (exact PDF, not stripped). Fees=Freight Charge - Wholesale - In 142.85 (Additional Charge Fees id 11, not PPV). PPV=0.30. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -781,7 +789,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 9/17/26 Legacy Wire (717)</t>
+          <t>TRANSFER AP (375)</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -791,7 +799,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>0.30</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -806,7 +814,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
@@ -835,7 +843,7 @@
       <c r="E6" s="2" t="n">
         <v>114.28</v>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>

</xml_diff>

<commit_message>
Enter Legacy Wire plus-5 on batch 717 and refresh the 9/17 sheet.
PS-INV104012 / 10124 Success (receipt 23647 2@100 + freight Fees).
104013 / 10123, 104011 / 10125, 104009 / 10127 HOLD missing receipt
(Ruben). 104010 / 10126 HOLD over-PPV $1.50 vs leftover $0.75 (Shawn;
receipts not selected). Keep 10112–10115 Success and 10116 HOLD.
NOTE-39 category/owner on every HOLD. invent=false. No Mail.Send.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-17-legacy-wire.xlsx
+++ b/runs/AP-run-2026-09-17-legacy-wire.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="AP run" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Exception counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$O$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -67,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -81,6 +82,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -446,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -456,14 +458,16 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -504,40 +508,50 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Exception category</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Exception owner</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>KIMCO id</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Batch</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Fees and surcharges</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>PPV</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Attach status</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Flag in Outlook</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Flag status</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -577,40 +591,42 @@
           <t>Finished bill (Invoice_Type 3). Header PO set=59034. Select Receipts 24187 19@41.0 on PO 59034. Invoice #=PS-INV104020 (exact PDF, not stripped). Fees=Freight Charge - Wholesale - In 250.0 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="n">
         <v>10112</v>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/17/26 Legacy Wire (717)</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Freight Charge - Wholesale - In 250.0</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>attached</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>entered-in-ai</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -646,40 +662,42 @@
           <t>Finished bill (Invoice_Type 3). Header PO set=59030. Select Receipts 24188 17@36.0; 24191 27@44.0 on PO 59030. Invoice #=PS-INV104019 (exact PDF, not stripped). Fees=Freight Charge - Wholesale - In 800.0 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="n">
         <v>10113</v>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/17/26 Legacy Wire (717)</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Freight Charge - Wholesale - In 800.0</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>attached</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>entered-in-ai</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -715,40 +733,42 @@
           <t>Finished bill (Invoice_Type 3). Header PO set=59030. Select Receipts 24189 9@41.0; 24190 17@41.0 on PO 59030. Invoice #=PS-INV104018 (exact PDF, not stripped). Fees=Freight Charge - Wholesale - In 371.42 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="n">
         <v>10114</v>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/17/26 Legacy Wire (717)</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Freight Charge - Wholesale - In 371.42</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>attached</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>entered-in-ai</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -784,40 +804,42 @@
           <t>Finished bill (Invoice_Type 3). Header PO set=58977. Select Receipts 24192 100@0.777 on PO 58977. Invoice #=PS-INV104015 (exact PDF, not stripped). Fees=Freight Charge - Wholesale - In 142.85 (Additional Charge Fees id 11, not PPV). PPV=0.30. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n">
         <v>10115</v>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>TRANSFER AP (375)</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Freight Charge - Wholesale - In 142.85</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>0.30</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>attached</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>entered-in-ai</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -850,46 +872,493 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="n">
+          <t>category=price_variance; owner=Shawn McKibben. HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>price_variance</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Shawn McKibben</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
         <v>10116</v>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/17/26 Legacy Wire (717)</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Freight Charge - Wholesale - In 14.28</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>attached</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>entered-with-issues</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Legacy Wire Products</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>PS-INV104013</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>58748</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>315.9</v>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 58748 for Legacy Wire invoice #PS-INV104013. PDF merch=A-05480-001 3@100; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Ruben Perez</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>10123</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Legacy Wire (717)</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Freight Charge - Wholesale - In 15.9</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Legacy Wire Products</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>PS-INV104012</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>58717</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>210.6</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 3). Header PO set=58717. Select Receipts 23647 2@100.0 on PO 58717. Invoice #=PS-INV104012 (exact PDF, not stripped). Fees=Freight Charge - Wholesale - In 10.6 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[{'id': 23647, 'qty': 2.0}] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="n">
+        <v>10124</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Legacy Wire (717)</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Freight Charge - Wholesale - In 10.6</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Legacy Wire Products</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>PS-INV104011</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>59063</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>875</v>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59063 for Legacy Wire invoice #PS-INV104011. PDF merch=Excl. Tax KANNON- WIF-10180 WIF-10180 Hitch Bolt Mirror Jet Black 09/01/26 25@35; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Ruben Perez</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>10125</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Legacy Wire (717)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Legacy Wire Products</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>PS-INV104010</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>59008</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>1195.5</v>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>category=price_variance; owner=Shawn McKibben. HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>price_variance</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Shawn McKibben</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>10126</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Legacy Wire (717)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Legacy Wire Products</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>PS-INV104009</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>58973</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 58973 for Legacy Wire invoice #PS-INV104009. PDF merch=Excl. Tax KANNON- MD20-1627 MD20-1627 BRACKET:  BK08 PFB735S2 FLAT BLACK 08/19/2 100@0.75; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Ruben Perez</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>10127</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/17/26 Legacy Wire (717)</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O6"/>
+  <autoFilter ref="A1:Q11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Exception category</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>price_variance</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record live Success for Legacy Wire 10126 on batch 717.
Select Receipts 24207/24208/24209 at $1.50; Invoice_Amount $1,195.50;
Outlook Entered in AI. No Transfer AP, no PPV, no Mail.Send.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-17-legacy-wire.xlsx
+++ b/runs/AP-run-2026-09-17-legacy-wire.xlsx
@@ -1157,7 +1157,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PS-INV104010</t>
+          <t>PS-INV104009</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1167,11 +1167,11 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>59008</t>
+          <t>58973</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>1195.5</v>
+        <v>75</v>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
@@ -1180,21 +1180,21 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>category=price_variance; owner=Shawn McKibben. HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 58973 for Legacy Wire invoice #PS-INV104009. PDF merch=Excl. Tax KANNON- MD20-1627 MD20-1627 BRACKET:  BK08 PFB735S2 FLAT BLACK 08/19/2 100@0.75; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>price_variance</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Shawn McKibben</t>
+          <t>Ruben Perez</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>10126</v>
+        <v>10127</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>PS-INV104009</t>
+          <t>PS-INV104010</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1246,34 +1246,26 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>58973</t>
+          <t>59008</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>1195.5</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 58973 for Legacy Wire invoice #PS-INV104009. PDF merch=Excl. Tax KANNON- MD20-1627 MD20-1627 BRACKET:  BK08 PFB735S2 FLAT BLACK 08/19/2 100@0.75; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59008. Select Receipts 24207 299@1.5; 24208 199@1.5; 24209 299@1.5 on PO 59008. Invoice #=PS-INV104010 (exact PDF, not stripped). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24207, 24208, 24209] fees=none ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="n">
-        <v>10127</v>
+        <v>10126</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
@@ -1302,7 +1294,7 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr"/>
@@ -1355,7 +1347,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh the 9/17 Legacy Wire sheet after HOLD receipts finished.
All four prior HOLDs (104017/104013/104011/104009) selected 9/18 leftovers and finished Success on batch 717. No Transfer AP; no Mail.Send.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-17-legacy-wire.xlsx
+++ b/runs/AP-run-2026-09-17-legacy-wire.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -50,11 +50,6 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -68,7 +63,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -77,9 +72,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -849,7 +841,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>PS-INV104017</t>
+          <t>PS-INV104012</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -859,34 +851,26 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>58807</t>
+          <t>58717</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>114.28</v>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>210.6</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>category=price_variance; owner=Shawn McKibben. HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>price_variance</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Shawn McKibben</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=58717. Select Receipts 23647 2@100.0 on PO 58717. Invoice #=PS-INV104012 (exact PDF, not stripped). Fees=Freight Charge - Wholesale - In 10.6 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[{'id': 23647, 'qty': 2.0}] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="n">
-        <v>10116</v>
+        <v>10124</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
@@ -895,7 +879,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Freight Charge - Wholesale - In 14.28</t>
+          <t>Freight Charge - Wholesale - In 10.6</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -915,7 +899,7 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr"/>
@@ -928,44 +912,36 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>PS-INV104013</t>
+          <t>PS-INV104010</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>58748</t>
+          <t>59008</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>315.9</v>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>1195.5</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 58748 for Legacy Wire invoice #PS-INV104013. PDF merch=A-05480-001 3@100; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59008. Select Receipts 24207 299@1.5; 24208 199@1.5; 24209 299@1.5 on PO 59008. Invoice #=PS-INV104010 (exact PDF, not stripped). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24207, 24208, 24209] fees=none ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="n">
-        <v>10123</v>
+        <v>10126</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
@@ -974,7 +950,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Freight Charge - Wholesale - In 15.9</t>
+          <t>none</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -994,7 +970,7 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr"/>
@@ -1007,7 +983,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>PS-INV104012</t>
+          <t>PS-INV104017</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1017,11 +993,11 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>58717</t>
+          <t>58807</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>210.6</v>
+        <v>114.28</v>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
@@ -1030,13 +1006,13 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 3). Header PO set=58717. Select Receipts 23647 2@100.0 on PO 58717. Invoice #=PS-INV104012 (exact PDF, not stripped). Fees=Freight Charge - Wholesale - In 10.6 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[{'id': 23647, 'qty': 2.0}] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set=58807. Select Receipts 24220 1@100.0 on PO 58807. Invoice #=PS-INV104017 (exact PDF, not stripped). Fees=Freight Charge - Wholesale - In 14.28 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[{'id': 24220, 'qty': 1.0}] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="n">
-        <v>10124</v>
+        <v>10116</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
@@ -1045,7 +1021,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Freight Charge - Wholesale - In 10.6</t>
+          <t>Freight Charge - Wholesale - In 14.28</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1078,44 +1054,36 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>PS-INV104011</t>
+          <t>PS-INV104013</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>59063</t>
+          <t>58748</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>875</v>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>315.9</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59063 for Legacy Wire invoice #PS-INV104011. PDF merch=Excl. Tax KANNON- WIF-10180 WIF-10180 Hitch Bolt Mirror Jet Black 09/01/26 25@35; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=58748. Select Receipts 24217 3@100.0 on PO 58748. Invoice #=PS-INV104013 (exact PDF, not stripped). Fees=Freight Charge - Wholesale - In 15.9 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24217] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="n">
-        <v>10125</v>
+        <v>10123</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
@@ -1124,14 +1092,14 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
+          <t>Freight Charge - Wholesale - In 15.9</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
           <t>none</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
           <t>attached</t>
@@ -1144,7 +1112,7 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr"/>
@@ -1157,7 +1125,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PS-INV104009</t>
+          <t>PS-INV104011</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1167,34 +1135,26 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>58973</t>
+          <t>59063</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>875</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 58973 for Legacy Wire invoice #PS-INV104009. PDF merch=Excl. Tax KANNON- MD20-1627 MD20-1627 BRACKET:  BK08 PFB735S2 FLAT BLACK 08/19/2 100@0.75; selected=none. Do not first-open guess. Do not invent Success. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59063. Select Receipts 24218 25@35.0 on PO 59063. Invoice #=PS-INV104011 (exact PDF, not stripped). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24218] fees=none ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="n">
-        <v>10127</v>
+        <v>10125</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -1223,7 +1183,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr"/>
@@ -1236,7 +1196,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>PS-INV104010</t>
+          <t>PS-INV104009</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1246,11 +1206,11 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>59008</t>
+          <t>58973</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>1195.5</v>
+        <v>75</v>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
@@ -1259,13 +1219,13 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 3). Header PO set=59008. Select Receipts 24207 299@1.5; 24208 199@1.5; 24209 299@1.5 on PO 59008. Invoice #=PS-INV104010 (exact PDF, not stripped). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24207, 24208, 24209] fees=none ppv=none. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set=58973. Select Receipts 24219 100@0.75 on PO 58973. Invoice #=PS-INV104009 (exact PDF, not stripped). Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24219] fees=none ppv=none. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="n">
-        <v>10126</v>
+        <v>10127</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
@@ -1311,7 +1271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1319,35 +1279,15 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Exception category</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>price_variance</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>